<commit_message>
feat: 상자·소모품 분류를 ItemType.Box·Consumable로 옮기고 Special을 비운다 (T-150)
</commit_message>
<xml_diff>
--- a/GameDesign/Excel/Enum.xlsx
+++ b/GameDesign/Excel/Enum.xlsx
@@ -694,12 +694,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5546875" defaultRowHeight="17.25"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -854,7 +854,37 @@
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>특수</t>
+          <t>사용 안 함 (2026-10-12 상자·소모품을 Box·Consumable로 옮김 — 등급 Special과 겹침)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>상자</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>Consumable</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>소모품</t>
         </is>
       </c>
     </row>

</xml_diff>